<commit_message>
usuario pedido y carrito
</commit_message>
<xml_diff>
--- a/bd/usuarios.xlsx
+++ b/bd/usuarios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -595,6 +595,36 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>2026-02-20 15:47:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tatiana</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-02-25 13:46:04</t>
         </is>
       </c>
     </row>

</xml_diff>